<commit_message>
chore: sync spec gates, docs, and readiness artifacts
</commit_message>
<xml_diff>
--- a/docs/references/CS_AI_CHATBOT_DB.xlsx
+++ b/docs/references/CS_AI_CHATBOT_DB.xlsx
@@ -23207,7 +23207,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>-</t>
@@ -23218,7 +23217,6 @@
           <t>Requested user ID</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -23236,7 +23234,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>PENDING</t>
@@ -23269,7 +23266,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>json</t>
@@ -23302,7 +23298,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>-</t>
@@ -23313,7 +23308,6 @@
           <t>Range start UTC</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -23331,7 +23325,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>-</t>
@@ -23342,7 +23335,6 @@
           <t>Range end UTC</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -23360,7 +23352,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>1000</t>
@@ -23393,7 +23384,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>5242880</t>
@@ -23404,7 +23394,6 @@
           <t>Max payload bytes</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -23422,7 +23411,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>30</t>
@@ -23433,7 +23421,6 @@
           <t>Max processing duration(sec)</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -23451,7 +23438,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>0</t>
@@ -23462,7 +23448,6 @@
           <t>Exported row count</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -23480,7 +23465,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>0</t>
@@ -23491,7 +23475,6 @@
           <t>Exported total bytes</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -23509,7 +23492,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>-</t>
@@ -23520,7 +23502,6 @@
           <t>Failure code</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -23538,7 +23519,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>-</t>
@@ -23549,7 +23529,6 @@
           <t>Failure detail</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -23567,7 +23546,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>-</t>
@@ -23600,7 +23578,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>-</t>
@@ -23633,7 +23610,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>CURRENT_TIMESTAMP</t>
@@ -23644,7 +23620,6 @@
           <t>Created at UTC</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -23662,7 +23637,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>-</t>
@@ -23673,7 +23647,6 @@
           <t>Worker started at UTC</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -23691,7 +23664,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>-</t>
@@ -23702,7 +23674,6 @@
           <t>Completed at UTC</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23830,7 +23801,6 @@
           <t>Chunk order</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -23848,7 +23818,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>-</t>
@@ -23881,7 +23850,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>-</t>
@@ -23892,7 +23860,6 @@
           <t>Chunk SHA-256</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -23910,7 +23877,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>CURRENT_TIMESTAMP</t>
@@ -23921,7 +23887,6 @@
           <t>Created at UTC</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24012,7 +23977,6 @@
           <t>Scheduler lock key</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -24030,7 +23994,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>-</t>
@@ -24041,7 +24004,6 @@
           <t>Lock owner instance ID</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -24059,7 +24021,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>-</t>
@@ -24070,7 +24031,6 @@
           <t>Lease expiration UTC</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -24088,7 +24048,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>0</t>
@@ -24121,7 +24080,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>-</t>
@@ -24154,7 +24112,6 @@
           <t>NULL</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>-</t>
@@ -24187,7 +24144,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>0</t>
@@ -24220,7 +24176,6 @@
           <t>NOT NULL</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>CURRENT_TIMESTAMP</t>
@@ -24231,7 +24186,6 @@
           <t>Updated at UTC</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>